<commit_message>
scan: seg7 2026-08-14 18:15 CST
</commit_message>
<xml_diff>
--- a/output/full_scan/batch_seq8_2026-08-14.xlsx
+++ b/output/full_scan/batch_seq8_2026-08-14.xlsx
@@ -428,7 +428,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O128"/>
+  <dimension ref="A1:O129"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -4184,21 +4184,21 @@
     </row>
     <row r="71">
       <c r="A71" s="2" t="n">
-        <v>6944</v>
+        <v>7828</v>
       </c>
       <c r="B71" s="2" t="inlineStr">
         <is>
-          <t>兆聯實業</t>
+          <t>創新服務</t>
         </is>
       </c>
       <c r="C71" s="2" t="n">
         <v/>
       </c>
       <c r="D71" s="2" t="n">
-        <v>305.5036158603635</v>
+        <v>309.2427315002466</v>
       </c>
       <c r="E71" s="2" t="n">
-        <v>741</v>
+        <v>1720</v>
       </c>
       <c r="F71" s="2" t="inlineStr">
         <is>
@@ -4209,49 +4209,49 @@
         <v>0</v>
       </c>
       <c r="H71" s="2" t="n">
-        <v>38.89557605464912</v>
+        <v>49.91013823352073</v>
       </c>
       <c r="I71" s="2" t="n">
-        <v>23.70048025042467</v>
+        <v>13.28744016352874</v>
       </c>
       <c r="J71" s="2" t="n">
-        <v>0.340731473665198</v>
+        <v>0.8660790362484729</v>
       </c>
       <c r="K71" s="2" t="n">
         <v>0</v>
       </c>
       <c r="L71" s="2" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="M71" s="2" t="n">
         <v>-1</v>
       </c>
       <c r="N71" s="2" t="n">
-        <v>3.544138638083346</v>
+        <v>31.0479094990002</v>
       </c>
       <c r="O71" s="2" t="inlineStr">
         <is>
-          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, liquidity_ok, adx_trending</t>
+          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, liquidity_ok, obv_uptrend</t>
         </is>
       </c>
     </row>
     <row r="72">
       <c r="A72" s="2" t="n">
-        <v>7768</v>
+        <v>6944</v>
       </c>
       <c r="B72" s="2" t="inlineStr">
         <is>
-          <t>頌勝科技</t>
+          <t>兆聯實業</t>
         </is>
       </c>
       <c r="C72" s="2" t="n">
         <v/>
       </c>
       <c r="D72" s="2" t="n">
-        <v>303.7518549477656</v>
+        <v>305.5036158603635</v>
       </c>
       <c r="E72" s="2" t="n">
-        <v>267</v>
+        <v>741</v>
       </c>
       <c r="F72" s="2" t="inlineStr">
         <is>
@@ -4262,13 +4262,13 @@
         <v>0</v>
       </c>
       <c r="H72" s="2" t="n">
-        <v>41.9768841371916</v>
+        <v>38.89557605464912</v>
       </c>
       <c r="I72" s="2" t="n">
-        <v>40.69041020097538</v>
+        <v>23.70048025042467</v>
       </c>
       <c r="J72" s="2" t="n">
-        <v>0.863345301601242</v>
+        <v>0.340731473665198</v>
       </c>
       <c r="K72" s="2" t="n">
         <v>0</v>
@@ -4280,31 +4280,31 @@
         <v>-1</v>
       </c>
       <c r="N72" s="2" t="n">
-        <v>4.955809984411502</v>
+        <v>3.544138638083346</v>
       </c>
       <c r="O72" s="2" t="inlineStr">
         <is>
-          <t>market_above_ma60, avoid_chase, adx_trending, obv_uptrend</t>
+          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, liquidity_ok, adx_trending</t>
         </is>
       </c>
     </row>
     <row r="73">
       <c r="A73" s="2" t="n">
-        <v>7820</v>
+        <v>7768</v>
       </c>
       <c r="B73" s="2" t="inlineStr">
         <is>
-          <t>立盈</t>
+          <t>頌勝科技</t>
         </is>
       </c>
       <c r="C73" s="2" t="n">
         <v/>
       </c>
       <c r="D73" s="2" t="n">
-        <v>298.5651342040363</v>
+        <v>303.7518549477656</v>
       </c>
       <c r="E73" s="2" t="n">
-        <v>120</v>
+        <v>267</v>
       </c>
       <c r="F73" s="2" t="inlineStr">
         <is>
@@ -4315,13 +4315,13 @@
         <v>0</v>
       </c>
       <c r="H73" s="2" t="n">
-        <v>60.78330438225703</v>
+        <v>41.9768841371916</v>
       </c>
       <c r="I73" s="2" t="n">
-        <v>21.46706787537452</v>
+        <v>40.69041020097538</v>
       </c>
       <c r="J73" s="2" t="n">
-        <v>2.64641383356119</v>
+        <v>0.863345301601242</v>
       </c>
       <c r="K73" s="2" t="n">
         <v>0</v>
@@ -4333,31 +4333,31 @@
         <v>-1</v>
       </c>
       <c r="N73" s="2" t="n">
-        <v>2.836530325583484</v>
+        <v>4.955809984411502</v>
       </c>
       <c r="O73" s="2" t="inlineStr">
         <is>
-          <t>volume_break, rsi_strong, market_above_ma60, adx_trending</t>
+          <t>market_above_ma60, avoid_chase, adx_trending, obv_uptrend</t>
         </is>
       </c>
     </row>
     <row r="74">
       <c r="A74" s="2" t="n">
-        <v>7736</v>
+        <v>7820</v>
       </c>
       <c r="B74" s="2" t="inlineStr">
         <is>
-          <t>虎山</t>
+          <t>立盈</t>
         </is>
       </c>
       <c r="C74" s="2" t="n">
         <v/>
       </c>
       <c r="D74" s="2" t="n">
-        <v>295.9147799121743</v>
+        <v>298.5651342040363</v>
       </c>
       <c r="E74" s="2" t="n">
-        <v>71.3</v>
+        <v>120</v>
       </c>
       <c r="F74" s="2" t="inlineStr">
         <is>
@@ -4368,13 +4368,13 @@
         <v>0</v>
       </c>
       <c r="H74" s="2" t="n">
-        <v>57.29775591547128</v>
+        <v>60.78330438225703</v>
       </c>
       <c r="I74" s="2" t="n">
-        <v>16.40881221313612</v>
+        <v>21.46706787537452</v>
       </c>
       <c r="J74" s="2" t="n">
-        <v>0.8392864204480691</v>
+        <v>2.64641383356119</v>
       </c>
       <c r="K74" s="2" t="n">
         <v>0</v>
@@ -4386,31 +4386,31 @@
         <v>-1</v>
       </c>
       <c r="N74" s="2" t="n">
-        <v>0.1182576895748804</v>
+        <v>2.836530325583484</v>
       </c>
       <c r="O74" s="2" t="inlineStr">
         <is>
-          <t>rsi_strong, breakout_20d, market_above_ma60, avoid_chase, bb_squeeze_breakout</t>
+          <t>volume_break, rsi_strong, market_above_ma60, adx_trending</t>
         </is>
       </c>
     </row>
     <row r="75">
       <c r="A75" s="2" t="n">
-        <v>6955</v>
+        <v>7736</v>
       </c>
       <c r="B75" s="2" t="inlineStr">
         <is>
-          <t>邦睿生技-創</t>
+          <t>虎山</t>
         </is>
       </c>
       <c r="C75" s="2" t="n">
         <v/>
       </c>
       <c r="D75" s="2" t="n">
-        <v>295.5159108852196</v>
+        <v>295.9147799121743</v>
       </c>
       <c r="E75" s="2" t="n">
-        <v>123</v>
+        <v>71.3</v>
       </c>
       <c r="F75" s="2" t="inlineStr">
         <is>
@@ -4421,13 +4421,13 @@
         <v>0</v>
       </c>
       <c r="H75" s="2" t="n">
-        <v>52.09281140275635</v>
+        <v>57.29775591547128</v>
       </c>
       <c r="I75" s="2" t="n">
-        <v>9.362299067915274</v>
+        <v>16.40881221313612</v>
       </c>
       <c r="J75" s="2" t="n">
-        <v>1.166547409961187</v>
+        <v>0.8392864204480691</v>
       </c>
       <c r="K75" s="2" t="n">
         <v>0</v>
@@ -4439,31 +4439,31 @@
         <v>-1</v>
       </c>
       <c r="N75" s="2" t="n">
-        <v>2.542679869028796</v>
+        <v>0.1182576895748804</v>
       </c>
       <c r="O75" s="2" t="inlineStr">
         <is>
-          <t>market_above_ma60, avoid_chase, obv_uptrend, mfi_strong, above_ichimoku_cloud</t>
+          <t>rsi_strong, breakout_20d, market_above_ma60, avoid_chase, bb_squeeze_breakout</t>
         </is>
       </c>
     </row>
     <row r="76">
       <c r="A76" s="2" t="n">
-        <v>6936</v>
+        <v>6955</v>
       </c>
       <c r="B76" s="2" t="inlineStr">
         <is>
-          <t>永鴻生技</t>
+          <t>邦睿生技-創</t>
         </is>
       </c>
       <c r="C76" s="2" t="n">
         <v/>
       </c>
       <c r="D76" s="2" t="n">
-        <v>284.9533843035726</v>
+        <v>295.5159108852196</v>
       </c>
       <c r="E76" s="2" t="n">
-        <v>32.05</v>
+        <v>123</v>
       </c>
       <c r="F76" s="2" t="inlineStr">
         <is>
@@ -4474,13 +4474,13 @@
         <v>0</v>
       </c>
       <c r="H76" s="2" t="n">
-        <v>48.22400023094769</v>
+        <v>52.09281140275635</v>
       </c>
       <c r="I76" s="2" t="n">
-        <v>16.01371559889331</v>
+        <v>9.362299067915274</v>
       </c>
       <c r="J76" s="2" t="n">
-        <v>0.3703745489182903</v>
+        <v>1.166547409961187</v>
       </c>
       <c r="K76" s="2" t="n">
         <v>0</v>
@@ -4492,31 +4492,31 @@
         <v>-1</v>
       </c>
       <c r="N76" s="2" t="n">
-        <v>0.0852381714565823</v>
+        <v>2.542679869028796</v>
       </c>
       <c r="O76" s="2" t="inlineStr">
         <is>
-          <t>market_above_ma60, avoid_chase, obv_uptrend, mfi_strong</t>
+          <t>market_above_ma60, avoid_chase, obv_uptrend, mfi_strong, above_ichimoku_cloud</t>
         </is>
       </c>
     </row>
     <row r="77">
       <c r="A77" s="2" t="n">
-        <v>7712</v>
+        <v>6936</v>
       </c>
       <c r="B77" s="2" t="inlineStr">
         <is>
-          <t>博盛半導體</t>
+          <t>永鴻生技</t>
         </is>
       </c>
       <c r="C77" s="2" t="n">
         <v/>
       </c>
       <c r="D77" s="2" t="n">
-        <v>280.5062181326678</v>
+        <v>284.9533843035726</v>
       </c>
       <c r="E77" s="2" t="n">
-        <v>141.5</v>
+        <v>32.05</v>
       </c>
       <c r="F77" s="2" t="inlineStr">
         <is>
@@ -4527,16 +4527,16 @@
         <v>0</v>
       </c>
       <c r="H77" s="2" t="n">
-        <v>45.34613862191193</v>
+        <v>48.22400023094769</v>
       </c>
       <c r="I77" s="2" t="n">
-        <v>18.82756922244015</v>
+        <v>16.01371559889331</v>
       </c>
       <c r="J77" s="2" t="n">
-        <v>0.6168496989313502</v>
+        <v>0.3703745489182903</v>
       </c>
       <c r="K77" s="2" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="L77" s="2" t="n">
         <v>0</v>
@@ -4545,31 +4545,31 @@
         <v>-1</v>
       </c>
       <c r="N77" s="2" t="n">
-        <v>2.438168094316504</v>
+        <v>0.0852381714565823</v>
       </c>
       <c r="O77" s="2" t="inlineStr">
         <is>
-          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, mfi_strong</t>
+          <t>market_above_ma60, avoid_chase, obv_uptrend, mfi_strong</t>
         </is>
       </c>
     </row>
     <row r="78">
       <c r="A78" s="2" t="n">
-        <v>6910</v>
+        <v>7712</v>
       </c>
       <c r="B78" s="2" t="inlineStr">
         <is>
-          <t>德鴻</t>
+          <t>博盛半導體</t>
         </is>
       </c>
       <c r="C78" s="2" t="n">
         <v/>
       </c>
       <c r="D78" s="2" t="n">
-        <v>277.47120052014</v>
+        <v>280.5062181326678</v>
       </c>
       <c r="E78" s="2" t="n">
-        <v>24.1</v>
+        <v>141.5</v>
       </c>
       <c r="F78" s="2" t="inlineStr">
         <is>
@@ -4580,16 +4580,16 @@
         <v>0</v>
       </c>
       <c r="H78" s="2" t="n">
-        <v>35.90271046094797</v>
+        <v>45.34613862191193</v>
       </c>
       <c r="I78" s="2" t="n">
-        <v>22.6985184302452</v>
+        <v>18.82756922244015</v>
       </c>
       <c r="J78" s="2" t="n">
-        <v>2.585023143614116</v>
+        <v>0.6168496989313502</v>
       </c>
       <c r="K78" s="2" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L78" s="2" t="n">
         <v>0</v>
@@ -4598,31 +4598,31 @@
         <v>-1</v>
       </c>
       <c r="N78" s="2" t="n">
-        <v>0.1297648521804655</v>
+        <v>2.438168094316504</v>
       </c>
       <c r="O78" s="2" t="inlineStr">
         <is>
-          <t>volume_break, market_above_ma60, avoid_chase, adx_trending</t>
+          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, mfi_strong</t>
         </is>
       </c>
     </row>
     <row r="79">
       <c r="A79" s="2" t="n">
-        <v>6873</v>
+        <v>6910</v>
       </c>
       <c r="B79" s="2" t="inlineStr">
         <is>
-          <t>泓德能源</t>
+          <t>德鴻</t>
         </is>
       </c>
       <c r="C79" s="2" t="n">
         <v/>
       </c>
       <c r="D79" s="2" t="n">
-        <v>271.7605506470561</v>
+        <v>277.47120052014</v>
       </c>
       <c r="E79" s="2" t="n">
-        <v>69</v>
+        <v>24.1</v>
       </c>
       <c r="F79" s="2" t="inlineStr">
         <is>
@@ -4633,13 +4633,13 @@
         <v>0</v>
       </c>
       <c r="H79" s="2" t="n">
-        <v>27.95215047541689</v>
+        <v>35.90271046094797</v>
       </c>
       <c r="I79" s="2" t="n">
-        <v>21.50805714605085</v>
+        <v>22.6985184302452</v>
       </c>
       <c r="J79" s="2" t="n">
-        <v>1.576055064705614</v>
+        <v>2.585023143614116</v>
       </c>
       <c r="K79" s="2" t="n">
         <v>0</v>
@@ -4651,7 +4651,7 @@
         <v>-1</v>
       </c>
       <c r="N79" s="2" t="n">
-        <v>-0.9571892848454432</v>
+        <v>0.1297648521804655</v>
       </c>
       <c r="O79" s="2" t="inlineStr">
         <is>
@@ -4661,21 +4661,21 @@
     </row>
     <row r="80">
       <c r="A80" s="2" t="n">
-        <v>6967</v>
+        <v>6873</v>
       </c>
       <c r="B80" s="2" t="inlineStr">
         <is>
-          <t>汎瑋材料</t>
+          <t>泓德能源</t>
         </is>
       </c>
       <c r="C80" s="2" t="n">
         <v/>
       </c>
       <c r="D80" s="2" t="n">
-        <v>271.7024544209575</v>
+        <v>271.7605506470561</v>
       </c>
       <c r="E80" s="2" t="n">
-        <v>68.8</v>
+        <v>69</v>
       </c>
       <c r="F80" s="2" t="inlineStr">
         <is>
@@ -4686,16 +4686,16 @@
         <v>0</v>
       </c>
       <c r="H80" s="2" t="n">
-        <v>44.76751863961886</v>
+        <v>27.95215047541689</v>
       </c>
       <c r="I80" s="2" t="n">
-        <v>14.83820170451147</v>
+        <v>21.50805714605085</v>
       </c>
       <c r="J80" s="2" t="n">
-        <v>2.48207640213778</v>
+        <v>1.576055064705614</v>
       </c>
       <c r="K80" s="2" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="L80" s="2" t="n">
         <v>0</v>
@@ -4704,31 +4704,31 @@
         <v>-1</v>
       </c>
       <c r="N80" s="2" t="n">
-        <v>0.0221030548724358</v>
+        <v>-0.9571892848454432</v>
       </c>
       <c r="O80" s="2" t="inlineStr">
         <is>
-          <t>ema60_gt_ema120, volume_break, market_above_ma60, avoid_chase</t>
+          <t>volume_break, market_above_ma60, avoid_chase, adx_trending</t>
         </is>
       </c>
     </row>
     <row r="81">
       <c r="A81" s="2" t="n">
-        <v>7734</v>
+        <v>6967</v>
       </c>
       <c r="B81" s="2" t="inlineStr">
         <is>
-          <t>印能科技</t>
+          <t>汎瑋材料</t>
         </is>
       </c>
       <c r="C81" s="2" t="n">
         <v/>
       </c>
       <c r="D81" s="2" t="n">
-        <v>268.2627711845228</v>
+        <v>271.7024544209575</v>
       </c>
       <c r="E81" s="2" t="n">
-        <v>3090</v>
+        <v>68.8</v>
       </c>
       <c r="F81" s="2" t="inlineStr">
         <is>
@@ -4739,13 +4739,13 @@
         <v>0</v>
       </c>
       <c r="H81" s="2" t="n">
-        <v>45.32358806418704</v>
+        <v>44.76751863961886</v>
       </c>
       <c r="I81" s="2" t="n">
-        <v>9.331095282006494</v>
+        <v>14.83820170451147</v>
       </c>
       <c r="J81" s="2" t="n">
-        <v>0.68319592486936</v>
+        <v>2.48207640213778</v>
       </c>
       <c r="K81" s="2" t="n">
         <v>1</v>
@@ -4757,31 +4757,31 @@
         <v>-1</v>
       </c>
       <c r="N81" s="2" t="n">
-        <v>-25.88918844971895</v>
+        <v>0.0221030548724358</v>
       </c>
       <c r="O81" s="2" t="inlineStr">
         <is>
-          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, liquidity_ok</t>
+          <t>ema60_gt_ema120, volume_break, market_above_ma60, avoid_chase</t>
         </is>
       </c>
     </row>
     <row r="82">
       <c r="A82" s="2" t="n">
-        <v>6906</v>
+        <v>7734</v>
       </c>
       <c r="B82" s="2" t="inlineStr">
         <is>
-          <t>現觀科</t>
+          <t>印能科技</t>
         </is>
       </c>
       <c r="C82" s="2" t="n">
         <v/>
       </c>
       <c r="D82" s="2" t="n">
-        <v>267.9253952143391</v>
+        <v>268.2627711845228</v>
       </c>
       <c r="E82" s="2" t="n">
-        <v>73.7</v>
+        <v>3090</v>
       </c>
       <c r="F82" s="2" t="inlineStr">
         <is>
@@ -4792,16 +4792,16 @@
         <v>0</v>
       </c>
       <c r="H82" s="2" t="n">
-        <v>48.9012926972499</v>
+        <v>45.32358806418704</v>
       </c>
       <c r="I82" s="2" t="n">
-        <v>23.65183007294526</v>
+        <v>9.331095282006494</v>
       </c>
       <c r="J82" s="2" t="n">
-        <v>1.503335287500198</v>
+        <v>0.68319592486936</v>
       </c>
       <c r="K82" s="2" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L82" s="2" t="n">
         <v>0</v>
@@ -4810,31 +4810,31 @@
         <v>-1</v>
       </c>
       <c r="N82" s="2" t="n">
-        <v>1.071197965090938</v>
+        <v>-25.88918844971895</v>
       </c>
       <c r="O82" s="2" t="inlineStr">
         <is>
-          <t>volume_break, market_above_ma60, avoid_chase, adx_trending</t>
+          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, liquidity_ok</t>
         </is>
       </c>
     </row>
     <row r="83">
       <c r="A83" s="2" t="n">
-        <v>7823</v>
+        <v>6906</v>
       </c>
       <c r="B83" s="2" t="inlineStr">
         <is>
-          <t>奧義賽博-KY創</t>
+          <t>現觀科</t>
         </is>
       </c>
       <c r="C83" s="2" t="n">
         <v/>
       </c>
       <c r="D83" s="2" t="n">
-        <v>267.652622163226</v>
+        <v>267.9253952143391</v>
       </c>
       <c r="E83" s="2" t="n">
-        <v>84.8</v>
+        <v>73.7</v>
       </c>
       <c r="F83" s="2" t="inlineStr">
         <is>
@@ -4845,13 +4845,13 @@
         <v>0</v>
       </c>
       <c r="H83" s="2" t="n">
-        <v>54.42129681733108</v>
+        <v>48.9012926972499</v>
       </c>
       <c r="I83" s="2" t="n">
-        <v>16.37122817997058</v>
+        <v>23.65183007294526</v>
       </c>
       <c r="J83" s="2" t="n">
-        <v>2.022676507241196</v>
+        <v>1.503335287500198</v>
       </c>
       <c r="K83" s="2" t="n">
         <v>0</v>
@@ -4863,31 +4863,31 @@
         <v>-1</v>
       </c>
       <c r="N83" s="2" t="n">
-        <v>0.588219142307794</v>
+        <v>1.071197965090938</v>
       </c>
       <c r="O83" s="2" t="inlineStr">
         <is>
-          <t>volume_break, market_above_ma60, avoid_chase, mfi_strong</t>
+          <t>volume_break, market_above_ma60, avoid_chase, adx_trending</t>
         </is>
       </c>
     </row>
     <row r="84">
       <c r="A84" s="2" t="n">
-        <v>6965</v>
+        <v>7823</v>
       </c>
       <c r="B84" s="2" t="inlineStr">
         <is>
-          <t>中傑-KY</t>
+          <t>奧義賽博-KY創</t>
         </is>
       </c>
       <c r="C84" s="2" t="n">
         <v/>
       </c>
       <c r="D84" s="2" t="n">
-        <v>264.2587945743564</v>
+        <v>267.652622163226</v>
       </c>
       <c r="E84" s="2" t="n">
-        <v>75.90000000000001</v>
+        <v>84.8</v>
       </c>
       <c r="F84" s="2" t="inlineStr">
         <is>
@@ -4898,13 +4898,13 @@
         <v>0</v>
       </c>
       <c r="H84" s="2" t="n">
-        <v>41.39147494797866</v>
+        <v>54.42129681733108</v>
       </c>
       <c r="I84" s="2" t="n">
-        <v>32.3111643064038</v>
+        <v>16.37122817997058</v>
       </c>
       <c r="J84" s="2" t="n">
-        <v>0.6366142697496168</v>
+        <v>2.022676507241196</v>
       </c>
       <c r="K84" s="2" t="n">
         <v>0</v>
@@ -4916,31 +4916,31 @@
         <v>-1</v>
       </c>
       <c r="N84" s="2" t="n">
-        <v>-0.124696373465224</v>
+        <v>0.588219142307794</v>
       </c>
       <c r="O84" s="2" t="inlineStr">
         <is>
-          <t>market_above_ma60, avoid_chase, adx_trending, mfi_strong</t>
+          <t>volume_break, market_above_ma60, avoid_chase, mfi_strong</t>
         </is>
       </c>
     </row>
     <row r="85">
       <c r="A85" s="2" t="n">
-        <v>6969</v>
+        <v>6965</v>
       </c>
       <c r="B85" s="2" t="inlineStr">
         <is>
-          <t>成信實業*-創</t>
+          <t>中傑-KY</t>
         </is>
       </c>
       <c r="C85" s="2" t="n">
         <v/>
       </c>
       <c r="D85" s="2" t="n">
-        <v>262.1730056938086</v>
+        <v>264.2587945743564</v>
       </c>
       <c r="E85" s="2" t="n">
-        <v>31.4</v>
+        <v>75.90000000000001</v>
       </c>
       <c r="F85" s="2" t="inlineStr">
         <is>
@@ -4951,13 +4951,13 @@
         <v>0</v>
       </c>
       <c r="H85" s="2" t="n">
-        <v>50.24306845448985</v>
+        <v>41.39147494797866</v>
       </c>
       <c r="I85" s="2" t="n">
-        <v>19.07128803044126</v>
+        <v>32.3111643064038</v>
       </c>
       <c r="J85" s="2" t="n">
-        <v>0.2805710751532995</v>
+        <v>0.6366142697496168</v>
       </c>
       <c r="K85" s="2" t="n">
         <v>0</v>
@@ -4969,31 +4969,31 @@
         <v>-1</v>
       </c>
       <c r="N85" s="2" t="n">
-        <v>-0.2964451547306779</v>
+        <v>-0.124696373465224</v>
       </c>
       <c r="O85" s="2" t="inlineStr">
         <is>
-          <t>market_above_ma60, avoid_chase, mfi_strong, above_ichimoku_cloud</t>
+          <t>market_above_ma60, avoid_chase, adx_trending, mfi_strong</t>
         </is>
       </c>
     </row>
     <row r="86">
       <c r="A86" s="2" t="n">
-        <v>6862</v>
+        <v>6969</v>
       </c>
       <c r="B86" s="2" t="inlineStr">
         <is>
-          <t>三集瑞-KY</t>
+          <t>成信實業*-創</t>
         </is>
       </c>
       <c r="C86" s="2" t="n">
         <v/>
       </c>
       <c r="D86" s="2" t="n">
-        <v>256.2170581010446</v>
+        <v>262.1730056938086</v>
       </c>
       <c r="E86" s="2" t="n">
-        <v>142.5</v>
+        <v>31.4</v>
       </c>
       <c r="F86" s="2" t="inlineStr">
         <is>
@@ -5004,13 +5004,13 @@
         <v>0</v>
       </c>
       <c r="H86" s="2" t="n">
-        <v>43.28327692592895</v>
+        <v>50.24306845448985</v>
       </c>
       <c r="I86" s="2" t="n">
-        <v>17.3658915585627</v>
+        <v>19.07128803044126</v>
       </c>
       <c r="J86" s="2" t="n">
-        <v>0.6062396550027288</v>
+        <v>0.2805710751532995</v>
       </c>
       <c r="K86" s="2" t="n">
         <v>0</v>
@@ -5022,31 +5022,31 @@
         <v>-1</v>
       </c>
       <c r="N86" s="2" t="n">
-        <v>2.940732758057958</v>
+        <v>-0.2964451547306779</v>
       </c>
       <c r="O86" s="2" t="inlineStr">
         <is>
-          <t>market_above_ma60, avoid_chase, obv_uptrend, mfi_strong</t>
+          <t>market_above_ma60, avoid_chase, mfi_strong, above_ichimoku_cloud</t>
         </is>
       </c>
     </row>
     <row r="87">
       <c r="A87" s="2" t="n">
-        <v>8032</v>
+        <v>6862</v>
       </c>
       <c r="B87" s="2" t="inlineStr">
         <is>
-          <t>光菱</t>
+          <t>三集瑞-KY</t>
         </is>
       </c>
       <c r="C87" s="2" t="n">
         <v/>
       </c>
       <c r="D87" s="2" t="n">
-        <v>244.2821499943803</v>
+        <v>256.2170581010446</v>
       </c>
       <c r="E87" s="2" t="n">
-        <v>36.85</v>
+        <v>142.5</v>
       </c>
       <c r="F87" s="2" t="inlineStr">
         <is>
@@ -5057,13 +5057,13 @@
         <v>0</v>
       </c>
       <c r="H87" s="2" t="n">
-        <v>45.61548785600763</v>
+        <v>43.28327692592895</v>
       </c>
       <c r="I87" s="2" t="n">
-        <v>24.57842074897824</v>
+        <v>17.3658915585627</v>
       </c>
       <c r="J87" s="2" t="n">
-        <v>0.8949460533787621</v>
+        <v>0.6062396550027288</v>
       </c>
       <c r="K87" s="2" t="n">
         <v>0</v>
@@ -5075,31 +5075,31 @@
         <v>-1</v>
       </c>
       <c r="N87" s="2" t="n">
-        <v>0.4747614836548435</v>
+        <v>2.940732758057958</v>
       </c>
       <c r="O87" s="2" t="inlineStr">
         <is>
-          <t>market_above_ma60, avoid_chase, adx_trending</t>
+          <t>market_above_ma60, avoid_chase, obv_uptrend, mfi_strong</t>
         </is>
       </c>
     </row>
     <row r="88">
       <c r="A88" s="2" t="n">
-        <v>7839</v>
+        <v>8032</v>
       </c>
       <c r="B88" s="2" t="inlineStr">
         <is>
-          <t>達人網</t>
+          <t>光菱</t>
         </is>
       </c>
       <c r="C88" s="2" t="n">
         <v/>
       </c>
       <c r="D88" s="2" t="n">
-        <v>229.7742264141389</v>
+        <v>244.2821499943803</v>
       </c>
       <c r="E88" s="2" t="n">
-        <v>45.8</v>
+        <v>36.85</v>
       </c>
       <c r="F88" s="2" t="inlineStr">
         <is>
@@ -5110,16 +5110,16 @@
         <v>0</v>
       </c>
       <c r="H88" s="2" t="n">
-        <v>49.3962570389249</v>
+        <v>45.61548785600763</v>
       </c>
       <c r="I88" s="2" t="n">
-        <v>15.7439743186985</v>
+        <v>24.57842074897824</v>
       </c>
       <c r="J88" s="2" t="n">
-        <v>1.24136090395901</v>
+        <v>0.8949460533787621</v>
       </c>
       <c r="K88" s="2" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="L88" s="2" t="n">
         <v>0</v>
@@ -5128,31 +5128,31 @@
         <v>-1</v>
       </c>
       <c r="N88" s="2" t="n">
-        <v>0.2483868642388091</v>
+        <v>0.4747614836548435</v>
       </c>
       <c r="O88" s="2" t="inlineStr">
         <is>
-          <t>market_above_ma60, avoid_chase, obv_uptrend</t>
+          <t>market_above_ma60, avoid_chase, adx_trending</t>
         </is>
       </c>
     </row>
     <row r="89">
       <c r="A89" s="2" t="n">
-        <v>6953</v>
+        <v>7839</v>
       </c>
       <c r="B89" s="2" t="inlineStr">
         <is>
-          <t>家碩</t>
+          <t>達人網</t>
         </is>
       </c>
       <c r="C89" s="2" t="n">
         <v/>
       </c>
       <c r="D89" s="2" t="n">
-        <v>229.523880038869</v>
+        <v>229.7742264141389</v>
       </c>
       <c r="E89" s="2" t="n">
-        <v>222</v>
+        <v>45.8</v>
       </c>
       <c r="F89" s="2" t="inlineStr">
         <is>
@@ -5163,16 +5163,16 @@
         <v>0</v>
       </c>
       <c r="H89" s="2" t="n">
-        <v>51.62012955195805</v>
+        <v>49.3962570389249</v>
       </c>
       <c r="I89" s="2" t="n">
-        <v>10.13710148344523</v>
+        <v>15.7439743186985</v>
       </c>
       <c r="J89" s="2" t="n">
-        <v>0.5879258010118044</v>
+        <v>1.24136090395901</v>
       </c>
       <c r="K89" s="2" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="L89" s="2" t="n">
         <v>0</v>
@@ -5181,7 +5181,7 @@
         <v>-1</v>
       </c>
       <c r="N89" s="2" t="n">
-        <v>2.40134764807617</v>
+        <v>0.2483868642388091</v>
       </c>
       <c r="O89" s="2" t="inlineStr">
         <is>
@@ -5191,21 +5191,21 @@
     </row>
     <row r="90">
       <c r="A90" s="2" t="n">
-        <v>6994</v>
+        <v>6953</v>
       </c>
       <c r="B90" s="2" t="inlineStr">
         <is>
-          <t>富威電力</t>
+          <t>家碩</t>
         </is>
       </c>
       <c r="C90" s="2" t="n">
         <v/>
       </c>
       <c r="D90" s="2" t="n">
-        <v>229.496496724818</v>
+        <v>229.5238800388689</v>
       </c>
       <c r="E90" s="2" t="n">
-        <v>35.9</v>
+        <v>222</v>
       </c>
       <c r="F90" s="2" t="inlineStr">
         <is>
@@ -5216,13 +5216,13 @@
         <v>0</v>
       </c>
       <c r="H90" s="2" t="n">
-        <v>30.76962388196905</v>
+        <v>51.62012955195805</v>
       </c>
       <c r="I90" s="2" t="n">
-        <v>37.89233606731543</v>
+        <v>10.13710148344523</v>
       </c>
       <c r="J90" s="2" t="n">
-        <v>0.6253206512985445</v>
+        <v>0.5879258010118044</v>
       </c>
       <c r="K90" s="2" t="n">
         <v>0</v>
@@ -5234,31 +5234,31 @@
         <v>-1</v>
       </c>
       <c r="N90" s="2" t="n">
-        <v>0.3669633460207531</v>
+        <v>2.40134764807617</v>
       </c>
       <c r="O90" s="2" t="inlineStr">
         <is>
-          <t>market_above_ma60, avoid_chase, adx_trending</t>
+          <t>market_above_ma60, avoid_chase, obv_uptrend</t>
         </is>
       </c>
     </row>
     <row r="91">
       <c r="A91" s="2" t="n">
-        <v>7791</v>
+        <v>6994</v>
       </c>
       <c r="B91" s="2" t="inlineStr">
         <is>
-          <t>皇家可口</t>
+          <t>富威電力</t>
         </is>
       </c>
       <c r="C91" s="2" t="n">
         <v/>
       </c>
       <c r="D91" s="2" t="n">
-        <v>228.4504313903481</v>
+        <v>229.496496724818</v>
       </c>
       <c r="E91" s="2" t="n">
-        <v>57.3</v>
+        <v>35.9</v>
       </c>
       <c r="F91" s="2" t="inlineStr">
         <is>
@@ -5269,13 +5269,13 @@
         <v>0</v>
       </c>
       <c r="H91" s="2" t="n">
-        <v>20.61970571054943</v>
+        <v>30.76962388196905</v>
       </c>
       <c r="I91" s="2" t="n">
-        <v>30.31124505848605</v>
+        <v>37.89233606731543</v>
       </c>
       <c r="J91" s="2" t="n">
-        <v>0.9763688194551184</v>
+        <v>0.6253206512985445</v>
       </c>
       <c r="K91" s="2" t="n">
         <v>0</v>
@@ -5287,7 +5287,7 @@
         <v>-1</v>
       </c>
       <c r="N91" s="2" t="n">
-        <v>-0.1952516290533283</v>
+        <v>0.3669633460207531</v>
       </c>
       <c r="O91" s="2" t="inlineStr">
         <is>
@@ -5297,21 +5297,21 @@
     </row>
     <row r="92">
       <c r="A92" s="2" t="n">
-        <v>6854</v>
+        <v>7791</v>
       </c>
       <c r="B92" s="2" t="inlineStr">
         <is>
-          <t>錼創科技-KY創</t>
+          <t>皇家可口</t>
         </is>
       </c>
       <c r="C92" s="2" t="n">
         <v/>
       </c>
       <c r="D92" s="2" t="n">
-        <v>228.422789302908</v>
+        <v>228.4504313903481</v>
       </c>
       <c r="E92" s="2" t="n">
-        <v>92.40000000000001</v>
+        <v>57.3</v>
       </c>
       <c r="F92" s="2" t="inlineStr">
         <is>
@@ -5322,13 +5322,13 @@
         <v>0</v>
       </c>
       <c r="H92" s="2" t="n">
-        <v>36.21907015994336</v>
+        <v>20.61970571054943</v>
       </c>
       <c r="I92" s="2" t="n">
-        <v>36.22550707785342</v>
+        <v>30.31124505848605</v>
       </c>
       <c r="J92" s="2" t="n">
-        <v>0.4656066249845472</v>
+        <v>0.9763688194551184</v>
       </c>
       <c r="K92" s="2" t="n">
         <v>0</v>
@@ -5340,7 +5340,7 @@
         <v>-1</v>
       </c>
       <c r="N92" s="2" t="n">
-        <v>1.349937193846068</v>
+        <v>-0.1952516290533283</v>
       </c>
       <c r="O92" s="2" t="inlineStr">
         <is>
@@ -5350,21 +5350,21 @@
     </row>
     <row r="93">
       <c r="A93" s="2" t="n">
-        <v>7842</v>
+        <v>6854</v>
       </c>
       <c r="B93" s="2" t="inlineStr">
         <is>
-          <t>天能綠電</t>
+          <t>錼創科技-KY創</t>
         </is>
       </c>
       <c r="C93" s="2" t="n">
         <v/>
       </c>
       <c r="D93" s="2" t="n">
-        <v>227.3281010132862</v>
+        <v>228.422789302908</v>
       </c>
       <c r="E93" s="2" t="n">
-        <v>85</v>
+        <v>92.40000000000001</v>
       </c>
       <c r="F93" s="2" t="inlineStr">
         <is>
@@ -5375,13 +5375,13 @@
         <v>0</v>
       </c>
       <c r="H93" s="2" t="n">
-        <v>48.39483445267506</v>
+        <v>36.21907015994336</v>
       </c>
       <c r="I93" s="2" t="n">
-        <v>10.55380764769474</v>
+        <v>36.22550707785342</v>
       </c>
       <c r="J93" s="2" t="n">
-        <v>3.150801955884746</v>
+        <v>0.4656066249845472</v>
       </c>
       <c r="K93" s="2" t="n">
         <v>0</v>
@@ -5393,31 +5393,31 @@
         <v>-1</v>
       </c>
       <c r="N93" s="2" t="n">
-        <v>1.620685858268563</v>
+        <v>1.349937193846068</v>
       </c>
       <c r="O93" s="2" t="inlineStr">
         <is>
-          <t>volume_break, market_above_ma60, avoid_chase</t>
+          <t>market_above_ma60, avoid_chase, adx_trending</t>
         </is>
       </c>
     </row>
     <row r="94">
       <c r="A94" s="2" t="n">
-        <v>6951</v>
+        <v>7842</v>
       </c>
       <c r="B94" s="2" t="inlineStr">
         <is>
-          <t>青新-創</t>
+          <t>天能綠電</t>
         </is>
       </c>
       <c r="C94" s="2" t="n">
         <v/>
       </c>
       <c r="D94" s="2" t="n">
-        <v>223.6513243379277</v>
+        <v>227.3281010132862</v>
       </c>
       <c r="E94" s="2" t="n">
-        <v>71.5</v>
+        <v>85</v>
       </c>
       <c r="F94" s="2" t="inlineStr">
         <is>
@@ -5428,13 +5428,13 @@
         <v>0</v>
       </c>
       <c r="H94" s="2" t="n">
-        <v>40.62553428633458</v>
+        <v>48.39483445267506</v>
       </c>
       <c r="I94" s="2" t="n">
-        <v>32.28601980442735</v>
+        <v>10.55380764769474</v>
       </c>
       <c r="J94" s="2" t="n">
-        <v>0.654434226593899</v>
+        <v>3.150801955884746</v>
       </c>
       <c r="K94" s="2" t="n">
         <v>0</v>
@@ -5446,31 +5446,31 @@
         <v>-1</v>
       </c>
       <c r="N94" s="2" t="n">
-        <v>0.3566592340090007</v>
+        <v>1.620685858268563</v>
       </c>
       <c r="O94" s="2" t="inlineStr">
         <is>
-          <t>market_above_ma60, avoid_chase, adx_trending</t>
+          <t>volume_break, market_above_ma60, avoid_chase</t>
         </is>
       </c>
     </row>
     <row r="95">
       <c r="A95" s="2" t="n">
-        <v>6996</v>
+        <v>6951</v>
       </c>
       <c r="B95" s="2" t="inlineStr">
         <is>
-          <t>力領科技</t>
+          <t>青新-創</t>
         </is>
       </c>
       <c r="C95" s="2" t="n">
         <v/>
       </c>
       <c r="D95" s="2" t="n">
-        <v>221.6029081625076</v>
+        <v>223.6513243379277</v>
       </c>
       <c r="E95" s="2" t="n">
-        <v>174</v>
+        <v>71.5</v>
       </c>
       <c r="F95" s="2" t="inlineStr">
         <is>
@@ -5481,13 +5481,13 @@
         <v>0</v>
       </c>
       <c r="H95" s="2" t="n">
-        <v>44.22311370845979</v>
+        <v>40.62553428633458</v>
       </c>
       <c r="I95" s="2" t="n">
-        <v>16.71556810806395</v>
+        <v>32.28601980442735</v>
       </c>
       <c r="J95" s="2" t="n">
-        <v>1.276196280192671</v>
+        <v>0.654434226593899</v>
       </c>
       <c r="K95" s="2" t="n">
         <v>0</v>
@@ -5499,31 +5499,31 @@
         <v>-1</v>
       </c>
       <c r="N95" s="2" t="n">
-        <v>0.7754517753560251</v>
+        <v>0.3566592340090007</v>
       </c>
       <c r="O95" s="2" t="inlineStr">
         <is>
-          <t>ema60_gt_ema120, market_above_ma60, avoid_chase</t>
+          <t>market_above_ma60, avoid_chase, adx_trending</t>
         </is>
       </c>
     </row>
     <row r="96">
       <c r="A96" s="2" t="n">
-        <v>6909</v>
+        <v>6996</v>
       </c>
       <c r="B96" s="2" t="inlineStr">
         <is>
-          <t>創控</t>
+          <t>力領科技</t>
         </is>
       </c>
       <c r="C96" s="2" t="n">
         <v/>
       </c>
       <c r="D96" s="2" t="n">
-        <v>221.0523793320567</v>
+        <v>221.6029081625076</v>
       </c>
       <c r="E96" s="2" t="n">
-        <v>40.4</v>
+        <v>174</v>
       </c>
       <c r="F96" s="2" t="inlineStr">
         <is>
@@ -5534,13 +5534,13 @@
         <v>0</v>
       </c>
       <c r="H96" s="2" t="n">
-        <v>39.60486907444952</v>
+        <v>44.22311370845979</v>
       </c>
       <c r="I96" s="2" t="n">
-        <v>25.83926174765221</v>
+        <v>16.71556810806395</v>
       </c>
       <c r="J96" s="2" t="n">
-        <v>0.7205798313295002</v>
+        <v>1.276196280192671</v>
       </c>
       <c r="K96" s="2" t="n">
         <v>0</v>
@@ -5552,31 +5552,31 @@
         <v>-1</v>
       </c>
       <c r="N96" s="2" t="n">
-        <v>0.4997545608901648</v>
+        <v>0.7754517753560251</v>
       </c>
       <c r="O96" s="2" t="inlineStr">
         <is>
-          <t>market_above_ma60, avoid_chase, adx_trending</t>
+          <t>ema60_gt_ema120, market_above_ma60, avoid_chase</t>
         </is>
       </c>
     </row>
     <row r="97">
       <c r="A97" s="2" t="n">
-        <v>6869</v>
+        <v>6909</v>
       </c>
       <c r="B97" s="2" t="inlineStr">
         <is>
-          <t>雲豹能源</t>
+          <t>創控</t>
         </is>
       </c>
       <c r="C97" s="2" t="n">
         <v/>
       </c>
       <c r="D97" s="2" t="n">
-        <v>220.2371207705689</v>
+        <v>221.0523793320567</v>
       </c>
       <c r="E97" s="2" t="n">
-        <v>64.09999999999999</v>
+        <v>40.4</v>
       </c>
       <c r="F97" s="2" t="inlineStr">
         <is>
@@ -5587,13 +5587,13 @@
         <v>0</v>
       </c>
       <c r="H97" s="2" t="n">
-        <v>36.01441114006797</v>
+        <v>39.60486907444952</v>
       </c>
       <c r="I97" s="2" t="n">
-        <v>16.30221249588943</v>
+        <v>25.83926174765221</v>
       </c>
       <c r="J97" s="2" t="n">
-        <v>0.981000313210352</v>
+        <v>0.7205798313295002</v>
       </c>
       <c r="K97" s="2" t="n">
         <v>0</v>
@@ -5605,31 +5605,31 @@
         <v>-1</v>
       </c>
       <c r="N97" s="2" t="n">
-        <v>0.1909704762970294</v>
+        <v>0.4997545608901648</v>
       </c>
       <c r="O97" s="2" t="inlineStr">
         <is>
-          <t>market_above_ma60, avoid_chase, obv_uptrend</t>
+          <t>market_above_ma60, avoid_chase, adx_trending</t>
         </is>
       </c>
     </row>
     <row r="98">
       <c r="A98" s="2" t="n">
-        <v>8028</v>
+        <v>6869</v>
       </c>
       <c r="B98" s="2" t="inlineStr">
         <is>
-          <t>昇陽半導體</t>
+          <t>雲豹能源</t>
         </is>
       </c>
       <c r="C98" s="2" t="n">
         <v/>
       </c>
       <c r="D98" s="2" t="n">
-        <v>217.5417203592398</v>
+        <v>220.2371207705689</v>
       </c>
       <c r="E98" s="2" t="n">
-        <v>263</v>
+        <v>64.09999999999999</v>
       </c>
       <c r="F98" s="2" t="inlineStr">
         <is>
@@ -5640,13 +5640,13 @@
         <v>0</v>
       </c>
       <c r="H98" s="2" t="n">
-        <v>44.62416922409719</v>
+        <v>36.01441114006797</v>
       </c>
       <c r="I98" s="2" t="n">
-        <v>16.82929040449758</v>
+        <v>16.30221249588943</v>
       </c>
       <c r="J98" s="2" t="n">
-        <v>1.493496429508654</v>
+        <v>0.981000313210352</v>
       </c>
       <c r="K98" s="2" t="n">
         <v>0</v>
@@ -5658,31 +5658,31 @@
         <v>-1</v>
       </c>
       <c r="N98" s="2" t="n">
-        <v>0.3427826548737407</v>
+        <v>0.1909704762970294</v>
       </c>
       <c r="O98" s="2" t="inlineStr">
         <is>
-          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, liquidity_ok</t>
+          <t>market_above_ma60, avoid_chase, obv_uptrend</t>
         </is>
       </c>
     </row>
     <row r="99">
       <c r="A99" s="2" t="n">
-        <v>7749</v>
+        <v>8028</v>
       </c>
       <c r="B99" s="2" t="inlineStr">
         <is>
-          <t>意騰-KY</t>
+          <t>昇陽半導體</t>
         </is>
       </c>
       <c r="C99" s="2" t="n">
         <v/>
       </c>
       <c r="D99" s="2" t="n">
-        <v>216.5051168069752</v>
+        <v>217.5417203592398</v>
       </c>
       <c r="E99" s="2" t="n">
-        <v>348.5</v>
+        <v>263</v>
       </c>
       <c r="F99" s="2" t="inlineStr">
         <is>
@@ -5693,13 +5693,13 @@
         <v>0</v>
       </c>
       <c r="H99" s="2" t="n">
-        <v>42.18782972305638</v>
+        <v>44.62416922409719</v>
       </c>
       <c r="I99" s="2" t="n">
-        <v>27.63450048585814</v>
+        <v>16.82929040449758</v>
       </c>
       <c r="J99" s="2" t="n">
-        <v>1.202070612450747</v>
+        <v>1.493496429508654</v>
       </c>
       <c r="K99" s="2" t="n">
         <v>0</v>
@@ -5711,31 +5711,31 @@
         <v>-1</v>
       </c>
       <c r="N99" s="2" t="n">
-        <v>6.308857573852958</v>
+        <v>0.3427826548737407</v>
       </c>
       <c r="O99" s="2" t="inlineStr">
         <is>
-          <t>market_above_ma60, avoid_chase, adx_trending</t>
+          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, liquidity_ok</t>
         </is>
       </c>
     </row>
     <row r="100">
       <c r="A100" s="2" t="n">
-        <v>6971</v>
+        <v>7749</v>
       </c>
       <c r="B100" s="2" t="inlineStr">
         <is>
-          <t>惠民實業</t>
+          <t>意騰-KY</t>
         </is>
       </c>
       <c r="C100" s="2" t="n">
         <v/>
       </c>
       <c r="D100" s="2" t="n">
-        <v>216.2009439655704</v>
+        <v>216.5051168069752</v>
       </c>
       <c r="E100" s="2" t="n">
-        <v>25.5</v>
+        <v>348.5</v>
       </c>
       <c r="F100" s="2" t="inlineStr">
         <is>
@@ -5746,16 +5746,16 @@
         <v>0</v>
       </c>
       <c r="H100" s="2" t="n">
-        <v>35.45171960876868</v>
+        <v>42.18782972305638</v>
       </c>
       <c r="I100" s="2" t="n">
-        <v>18.14273678172235</v>
+        <v>27.63450048585814</v>
       </c>
       <c r="J100" s="2" t="n">
-        <v>2.021566787416459</v>
+        <v>1.202070612450747</v>
       </c>
       <c r="K100" s="2" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="L100" s="2" t="n">
         <v>0</v>
@@ -5764,31 +5764,31 @@
         <v>-1</v>
       </c>
       <c r="N100" s="2" t="n">
-        <v>-0.0208395188718678</v>
+        <v>6.308857573852958</v>
       </c>
       <c r="O100" s="2" t="inlineStr">
         <is>
-          <t>volume_break, market_above_ma60, avoid_chase, kd_golden_cross</t>
+          <t>market_above_ma60, avoid_chase, adx_trending</t>
         </is>
       </c>
     </row>
     <row r="101">
       <c r="A101" s="2" t="n">
-        <v>8024</v>
+        <v>6971</v>
       </c>
       <c r="B101" s="2" t="inlineStr">
         <is>
-          <t>佑華</t>
+          <t>惠民實業</t>
         </is>
       </c>
       <c r="C101" s="2" t="n">
         <v/>
       </c>
       <c r="D101" s="2" t="n">
-        <v>216.0962536163265</v>
+        <v>216.2009439655704</v>
       </c>
       <c r="E101" s="2" t="n">
-        <v>13.6</v>
+        <v>25.5</v>
       </c>
       <c r="F101" s="2" t="inlineStr">
         <is>
@@ -5799,16 +5799,16 @@
         <v>0</v>
       </c>
       <c r="H101" s="2" t="n">
-        <v>40.55594826937073</v>
+        <v>35.45171960876868</v>
       </c>
       <c r="I101" s="2" t="n">
-        <v>14.71984008436988</v>
+        <v>18.14273678172235</v>
       </c>
       <c r="J101" s="2" t="n">
-        <v>0.8042849163595472</v>
+        <v>2.021566787416459</v>
       </c>
       <c r="K101" s="2" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L101" s="2" t="n">
         <v>0</v>
@@ -5817,31 +5817,31 @@
         <v>-1</v>
       </c>
       <c r="N101" s="2" t="n">
-        <v>-0.1255848427969196</v>
+        <v>-0.0208395188718678</v>
       </c>
       <c r="O101" s="2" t="inlineStr">
         <is>
-          <t>ema60_gt_ema120, market_above_ma60, avoid_chase</t>
+          <t>volume_break, market_above_ma60, avoid_chase, kd_golden_cross</t>
         </is>
       </c>
     </row>
     <row r="102">
       <c r="A102" s="2" t="n">
-        <v>6887</v>
+        <v>8024</v>
       </c>
       <c r="B102" s="2" t="inlineStr">
         <is>
-          <t>寶綠特-KY</t>
+          <t>佑華</t>
         </is>
       </c>
       <c r="C102" s="2" t="n">
         <v/>
       </c>
       <c r="D102" s="2" t="n">
-        <v>209.5006870702496</v>
+        <v>216.0962536163265</v>
       </c>
       <c r="E102" s="2" t="n">
-        <v>35.7</v>
+        <v>13.6</v>
       </c>
       <c r="F102" s="2" t="inlineStr">
         <is>
@@ -5852,13 +5852,13 @@
         <v>0</v>
       </c>
       <c r="H102" s="2" t="n">
-        <v>46.87480587345534</v>
+        <v>40.55594826937073</v>
       </c>
       <c r="I102" s="2" t="n">
-        <v>16.84127484109767</v>
+        <v>14.71984008436988</v>
       </c>
       <c r="J102" s="2" t="n">
-        <v>0.8563094976661513</v>
+        <v>0.8042849163595472</v>
       </c>
       <c r="K102" s="2" t="n">
         <v>0</v>
@@ -5870,31 +5870,31 @@
         <v>-1</v>
       </c>
       <c r="N102" s="2" t="n">
-        <v>-0.2094027687861783</v>
+        <v>-0.1255848427969196</v>
       </c>
       <c r="O102" s="2" t="inlineStr">
         <is>
-          <t>market_above_ma60, avoid_chase, above_ichimoku_cloud</t>
+          <t>ema60_gt_ema120, market_above_ma60, avoid_chase</t>
         </is>
       </c>
     </row>
     <row r="103">
       <c r="A103" s="2" t="n">
-        <v>6894</v>
+        <v>6887</v>
       </c>
       <c r="B103" s="2" t="inlineStr">
         <is>
-          <t>衛司特</t>
+          <t>寶綠特-KY</t>
         </is>
       </c>
       <c r="C103" s="2" t="n">
         <v/>
       </c>
       <c r="D103" s="2" t="n">
-        <v>209.1237729345333</v>
+        <v>209.5006870702496</v>
       </c>
       <c r="E103" s="2" t="n">
-        <v>336</v>
+        <v>35.7</v>
       </c>
       <c r="F103" s="2" t="inlineStr">
         <is>
@@ -5905,13 +5905,13 @@
         <v>0</v>
       </c>
       <c r="H103" s="2" t="n">
-        <v>47.85427182003508</v>
+        <v>46.87480587345534</v>
       </c>
       <c r="I103" s="2" t="n">
-        <v>13.33227243521672</v>
+        <v>16.84127484109767</v>
       </c>
       <c r="J103" s="2" t="n">
-        <v>0.5062683501345211</v>
+        <v>0.8563094976661513</v>
       </c>
       <c r="K103" s="2" t="n">
         <v>0</v>
@@ -5923,31 +5923,31 @@
         <v>-1</v>
       </c>
       <c r="N103" s="2" t="n">
-        <v>1.957458611015152</v>
+        <v>-0.2094027687861783</v>
       </c>
       <c r="O103" s="2" t="inlineStr">
         <is>
-          <t>ema60_gt_ema120, market_above_ma60, avoid_chase</t>
+          <t>market_above_ma60, avoid_chase, above_ichimoku_cloud</t>
         </is>
       </c>
     </row>
     <row r="104">
       <c r="A104" s="2" t="n">
-        <v>7780</v>
+        <v>6894</v>
       </c>
       <c r="B104" s="2" t="inlineStr">
         <is>
-          <t>大研生醫*</t>
+          <t>衛司特</t>
         </is>
       </c>
       <c r="C104" s="2" t="n">
         <v/>
       </c>
       <c r="D104" s="2" t="n">
-        <v>207.8504153614478</v>
+        <v>209.1237729345333</v>
       </c>
       <c r="E104" s="2" t="n">
-        <v>16.6</v>
+        <v>336</v>
       </c>
       <c r="F104" s="2" t="inlineStr">
         <is>
@@ -5958,13 +5958,13 @@
         <v>0</v>
       </c>
       <c r="H104" s="2" t="n">
-        <v>33.90868444723665</v>
+        <v>47.85427182003508</v>
       </c>
       <c r="I104" s="2" t="n">
-        <v>33.78673706953624</v>
+        <v>13.33227243521672</v>
       </c>
       <c r="J104" s="2" t="n">
-        <v>0.9656842984460962</v>
+        <v>0.5062683501345211</v>
       </c>
       <c r="K104" s="2" t="n">
         <v>0</v>
@@ -5976,31 +5976,31 @@
         <v>-1</v>
       </c>
       <c r="N104" s="2" t="n">
-        <v>0.0332198611407321</v>
+        <v>1.957458611015152</v>
       </c>
       <c r="O104" s="2" t="inlineStr">
         <is>
-          <t>market_above_ma60, avoid_chase, adx_trending</t>
+          <t>ema60_gt_ema120, market_above_ma60, avoid_chase</t>
         </is>
       </c>
     </row>
     <row r="105">
       <c r="A105" s="2" t="n">
-        <v>7818</v>
+        <v>7780</v>
       </c>
       <c r="B105" s="2" t="inlineStr">
         <is>
-          <t>溢泰實業</t>
+          <t>大研生醫*</t>
         </is>
       </c>
       <c r="C105" s="2" t="n">
         <v/>
       </c>
       <c r="D105" s="2" t="n">
-        <v>207.3223037754992</v>
+        <v>207.8504153614478</v>
       </c>
       <c r="E105" s="2" t="n">
-        <v>62.4</v>
+        <v>16.6</v>
       </c>
       <c r="F105" s="2" t="inlineStr">
         <is>
@@ -6011,13 +6011,13 @@
         <v>0</v>
       </c>
       <c r="H105" s="2" t="n">
-        <v>34.16045343358255</v>
+        <v>33.90868444723665</v>
       </c>
       <c r="I105" s="2" t="n">
-        <v>29.01094432035923</v>
+        <v>33.78673706953624</v>
       </c>
       <c r="J105" s="2" t="n">
-        <v>0.5856831593281888</v>
+        <v>0.9656842984460962</v>
       </c>
       <c r="K105" s="2" t="n">
         <v>0</v>
@@ -6029,7 +6029,7 @@
         <v>-1</v>
       </c>
       <c r="N105" s="2" t="n">
-        <v>-0.0738015234613713</v>
+        <v>0.0332198611407321</v>
       </c>
       <c r="O105" s="2" t="inlineStr">
         <is>
@@ -6039,21 +6039,21 @@
     </row>
     <row r="106">
       <c r="A106" s="2" t="n">
-        <v>8038</v>
+        <v>7818</v>
       </c>
       <c r="B106" s="2" t="inlineStr">
         <is>
-          <t>長園科</t>
+          <t>溢泰實業</t>
         </is>
       </c>
       <c r="C106" s="2" t="n">
         <v/>
       </c>
       <c r="D106" s="2" t="n">
-        <v>206.5268560556802</v>
+        <v>207.3223037754992</v>
       </c>
       <c r="E106" s="2" t="n">
-        <v>31.1</v>
+        <v>62.4</v>
       </c>
       <c r="F106" s="2" t="inlineStr">
         <is>
@@ -6064,16 +6064,16 @@
         <v>0</v>
       </c>
       <c r="H106" s="2" t="n">
-        <v>32.82367718306017</v>
+        <v>34.16045343358255</v>
       </c>
       <c r="I106" s="2" t="n">
-        <v>21.53475091435028</v>
+        <v>29.01094432035923</v>
       </c>
       <c r="J106" s="2" t="n">
-        <v>1.452425405722226</v>
+        <v>0.5856831593281888</v>
       </c>
       <c r="K106" s="2" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="L106" s="2" t="n">
         <v>0</v>
@@ -6082,7 +6082,7 @@
         <v>-1</v>
       </c>
       <c r="N106" s="2" t="n">
-        <v>0.1188724768336033</v>
+        <v>-0.0738015234613713</v>
       </c>
       <c r="O106" s="2" t="inlineStr">
         <is>
@@ -6092,21 +6092,21 @@
     </row>
     <row r="107">
       <c r="A107" s="2" t="n">
-        <v>7821</v>
+        <v>8038</v>
       </c>
       <c r="B107" s="2" t="inlineStr">
         <is>
-          <t>神數</t>
+          <t>長園科</t>
         </is>
       </c>
       <c r="C107" s="2" t="n">
         <v/>
       </c>
       <c r="D107" s="2" t="n">
-        <v>204.8501429707632</v>
+        <v>206.5268560556802</v>
       </c>
       <c r="E107" s="2" t="n">
-        <v>39.4</v>
+        <v>31.1</v>
       </c>
       <c r="F107" s="2" t="inlineStr">
         <is>
@@ -6117,16 +6117,16 @@
         <v>0</v>
       </c>
       <c r="H107" s="2" t="n">
-        <v>39.45093397581463</v>
+        <v>32.82367718306017</v>
       </c>
       <c r="I107" s="2" t="n">
-        <v>16.73533760837734</v>
+        <v>21.53475091435028</v>
       </c>
       <c r="J107" s="2" t="n">
-        <v>0.5590416052693974</v>
+        <v>1.452425405722226</v>
       </c>
       <c r="K107" s="2" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="L107" s="2" t="n">
         <v>0</v>
@@ -6135,31 +6135,31 @@
         <v>-1</v>
       </c>
       <c r="N107" s="2" t="n">
-        <v>0.0407701689867967</v>
+        <v>0.1188724768336033</v>
       </c>
       <c r="O107" s="2" t="inlineStr">
         <is>
-          <t>market_above_ma60, avoid_chase, obv_uptrend</t>
+          <t>market_above_ma60, avoid_chase, adx_trending</t>
         </is>
       </c>
     </row>
     <row r="108">
       <c r="A108" s="2" t="n">
-        <v>7770</v>
+        <v>7821</v>
       </c>
       <c r="B108" s="2" t="inlineStr">
         <is>
-          <t>君曜</t>
+          <t>神數</t>
         </is>
       </c>
       <c r="C108" s="2" t="n">
         <v/>
       </c>
       <c r="D108" s="2" t="n">
-        <v>203.6446213284129</v>
+        <v>204.8501429707632</v>
       </c>
       <c r="E108" s="2" t="n">
-        <v>39.75</v>
+        <v>39.4</v>
       </c>
       <c r="F108" s="2" t="inlineStr">
         <is>
@@ -6170,13 +6170,13 @@
         <v>0</v>
       </c>
       <c r="H108" s="2" t="n">
-        <v>52.28661558741754</v>
+        <v>39.45093397581463</v>
       </c>
       <c r="I108" s="2" t="n">
-        <v>10.96684684937829</v>
+        <v>16.73533760837734</v>
       </c>
       <c r="J108" s="2" t="n">
-        <v>0.3497945894345669</v>
+        <v>0.5590416052693974</v>
       </c>
       <c r="K108" s="2" t="n">
         <v>0</v>
@@ -6188,31 +6188,31 @@
         <v>-1</v>
       </c>
       <c r="N108" s="2" t="n">
-        <v>1.588629619054641</v>
+        <v>0.0407701689867967</v>
       </c>
       <c r="O108" s="2" t="inlineStr">
         <is>
-          <t>market_above_ma60, avoid_chase, obv_uptrend, mfi_strong</t>
+          <t>market_above_ma60, avoid_chase, obv_uptrend</t>
         </is>
       </c>
     </row>
     <row r="109">
       <c r="A109" s="2" t="n">
-        <v>6895</v>
+        <v>7770</v>
       </c>
       <c r="B109" s="2" t="inlineStr">
         <is>
-          <t>宏碩系統</t>
+          <t>君曜</t>
         </is>
       </c>
       <c r="C109" s="2" t="n">
         <v/>
       </c>
       <c r="D109" s="2" t="n">
-        <v>202.9038044725015</v>
+        <v>203.6446213284129</v>
       </c>
       <c r="E109" s="2" t="n">
-        <v>114.5</v>
+        <v>39.75</v>
       </c>
       <c r="F109" s="2" t="inlineStr">
         <is>
@@ -6223,13 +6223,13 @@
         <v>0</v>
       </c>
       <c r="H109" s="2" t="n">
-        <v>34.09061885506851</v>
+        <v>52.28661558741754</v>
       </c>
       <c r="I109" s="2" t="n">
-        <v>22.72537024548462</v>
+        <v>10.96684684937829</v>
       </c>
       <c r="J109" s="2" t="n">
-        <v>1.385843913806535</v>
+        <v>0.3497945894345669</v>
       </c>
       <c r="K109" s="2" t="n">
         <v>0</v>
@@ -6241,31 +6241,31 @@
         <v>-1</v>
       </c>
       <c r="N109" s="2" t="n">
-        <v>1.12312038849807</v>
+        <v>1.588629619054641</v>
       </c>
       <c r="O109" s="2" t="inlineStr">
         <is>
-          <t>market_above_ma60, avoid_chase, adx_trending</t>
+          <t>market_above_ma60, avoid_chase, obv_uptrend, mfi_strong</t>
         </is>
       </c>
     </row>
     <row r="110">
       <c r="A110" s="2" t="n">
-        <v>8034</v>
+        <v>6895</v>
       </c>
       <c r="B110" s="2" t="inlineStr">
         <is>
-          <t>榮群</t>
+          <t>宏碩系統</t>
         </is>
       </c>
       <c r="C110" s="2" t="n">
         <v/>
       </c>
       <c r="D110" s="2" t="n">
-        <v>202.5928390066647</v>
+        <v>202.9038044725015</v>
       </c>
       <c r="E110" s="2" t="n">
-        <v>18.8</v>
+        <v>114.5</v>
       </c>
       <c r="F110" s="2" t="inlineStr">
         <is>
@@ -6276,13 +6276,13 @@
         <v>0</v>
       </c>
       <c r="H110" s="2" t="n">
-        <v>37.18041414872728</v>
+        <v>34.09061885506851</v>
       </c>
       <c r="I110" s="2" t="n">
-        <v>36.32718468158631</v>
+        <v>22.72537024548462</v>
       </c>
       <c r="J110" s="2" t="n">
-        <v>1.255216141811082</v>
+        <v>1.385843913806535</v>
       </c>
       <c r="K110" s="2" t="n">
         <v>0</v>
@@ -6294,7 +6294,7 @@
         <v>-1</v>
       </c>
       <c r="N110" s="2" t="n">
-        <v>0.104654137184359</v>
+        <v>1.12312038849807</v>
       </c>
       <c r="O110" s="2" t="inlineStr">
         <is>
@@ -6304,21 +6304,21 @@
     </row>
     <row r="111">
       <c r="A111" s="2" t="n">
-        <v>6997</v>
+        <v>8034</v>
       </c>
       <c r="B111" s="2" t="inlineStr">
         <is>
-          <t>博弘</t>
+          <t>榮群</t>
         </is>
       </c>
       <c r="C111" s="2" t="n">
         <v/>
       </c>
       <c r="D111" s="2" t="n">
-        <v>200.8776903355902</v>
+        <v>202.5928390066647</v>
       </c>
       <c r="E111" s="2" t="n">
-        <v>69.3</v>
+        <v>18.8</v>
       </c>
       <c r="F111" s="2" t="inlineStr">
         <is>
@@ -6329,13 +6329,13 @@
         <v>0</v>
       </c>
       <c r="H111" s="2" t="n">
-        <v>52.65525582163289</v>
+        <v>37.18041414872728</v>
       </c>
       <c r="I111" s="2" t="n">
-        <v>11.19650550330738</v>
+        <v>36.32718468158631</v>
       </c>
       <c r="J111" s="2" t="n">
-        <v>0.2583127923939836</v>
+        <v>1.255216141811082</v>
       </c>
       <c r="K111" s="2" t="n">
         <v>0</v>
@@ -6347,31 +6347,31 @@
         <v>-1</v>
       </c>
       <c r="N111" s="2" t="n">
-        <v>-0.3678356072376143</v>
+        <v>0.104654137184359</v>
       </c>
       <c r="O111" s="2" t="inlineStr">
         <is>
-          <t>market_above_ma60, avoid_chase, williams_r_recovery, above_ichimoku_cloud</t>
+          <t>market_above_ma60, avoid_chase, adx_trending</t>
         </is>
       </c>
     </row>
     <row r="112">
       <c r="A112" s="2" t="n">
-        <v>7765</v>
+        <v>6997</v>
       </c>
       <c r="B112" s="2" t="inlineStr">
         <is>
-          <t>中華資安</t>
+          <t>博弘</t>
         </is>
       </c>
       <c r="C112" s="2" t="n">
         <v/>
       </c>
       <c r="D112" s="2" t="n">
-        <v>200.3134742472765</v>
+        <v>200.8776903355902</v>
       </c>
       <c r="E112" s="2" t="n">
-        <v>226.5</v>
+        <v>69.3</v>
       </c>
       <c r="F112" s="2" t="inlineStr">
         <is>
@@ -6382,13 +6382,13 @@
         <v>0</v>
       </c>
       <c r="H112" s="2" t="n">
-        <v>50.45792471943711</v>
+        <v>52.65525582163289</v>
       </c>
       <c r="I112" s="2" t="n">
-        <v>16.87513040760096</v>
+        <v>11.19650550330738</v>
       </c>
       <c r="J112" s="2" t="n">
-        <v>0.4225015046422413</v>
+        <v>0.2583127923939836</v>
       </c>
       <c r="K112" s="2" t="n">
         <v>0</v>
@@ -6400,31 +6400,31 @@
         <v>-1</v>
       </c>
       <c r="N112" s="2" t="n">
-        <v>0.7457980751366617</v>
+        <v>-0.3678356072376143</v>
       </c>
       <c r="O112" s="2" t="inlineStr">
         <is>
-          <t>market_above_ma60, avoid_chase, obv_uptrend</t>
+          <t>market_above_ma60, avoid_chase, williams_r_recovery, above_ichimoku_cloud</t>
         </is>
       </c>
     </row>
     <row r="113">
       <c r="A113" s="2" t="n">
-        <v>7803</v>
+        <v>7765</v>
       </c>
       <c r="B113" s="2" t="inlineStr">
         <is>
-          <t>雲象科技-創</t>
+          <t>中華資安</t>
         </is>
       </c>
       <c r="C113" s="2" t="n">
         <v/>
       </c>
       <c r="D113" s="2" t="n">
-        <v>191.0411350243054</v>
+        <v>200.3134742472765</v>
       </c>
       <c r="E113" s="2" t="n">
-        <v>19.7</v>
+        <v>226.5</v>
       </c>
       <c r="F113" s="2" t="inlineStr">
         <is>
@@ -6435,13 +6435,13 @@
         <v>0</v>
       </c>
       <c r="H113" s="2" t="n">
-        <v>39.27672906297025</v>
+        <v>50.45792471943711</v>
       </c>
       <c r="I113" s="2" t="n">
-        <v>19.91600029941464</v>
+        <v>16.87513040760096</v>
       </c>
       <c r="J113" s="2" t="n">
-        <v>0.3445841993981449</v>
+        <v>0.4225015046422413</v>
       </c>
       <c r="K113" s="2" t="n">
         <v>0</v>
@@ -6453,31 +6453,31 @@
         <v>-1</v>
       </c>
       <c r="N113" s="2" t="n">
-        <v>0.08479740408105201</v>
+        <v>0.7457980751366617</v>
       </c>
       <c r="O113" s="2" t="inlineStr">
         <is>
-          <t>market_above_ma60, avoid_chase, kd_golden_cross</t>
+          <t>market_above_ma60, avoid_chase, obv_uptrend</t>
         </is>
       </c>
     </row>
     <row r="114">
       <c r="A114" s="2" t="n">
-        <v>6908</v>
+        <v>7803</v>
       </c>
       <c r="B114" s="2" t="inlineStr">
         <is>
-          <t>宏碁遊戲-創</t>
+          <t>雲象科技-創</t>
         </is>
       </c>
       <c r="C114" s="2" t="n">
         <v/>
       </c>
       <c r="D114" s="2" t="n">
-        <v>183.0164824012788</v>
+        <v>191.0411350243054</v>
       </c>
       <c r="E114" s="2" t="n">
-        <v>32.8</v>
+        <v>19.7</v>
       </c>
       <c r="F114" s="2" t="inlineStr">
         <is>
@@ -6488,13 +6488,13 @@
         <v>0</v>
       </c>
       <c r="H114" s="2" t="n">
-        <v>38.25126317374618</v>
+        <v>39.27672906297025</v>
       </c>
       <c r="I114" s="2" t="n">
-        <v>31.2457795599022</v>
+        <v>19.91600029941464</v>
       </c>
       <c r="J114" s="2" t="n">
-        <v>0.2051535797206257</v>
+        <v>0.3445841993981449</v>
       </c>
       <c r="K114" s="2" t="n">
         <v>0</v>
@@ -6506,31 +6506,31 @@
         <v>-1</v>
       </c>
       <c r="N114" s="2" t="n">
-        <v>0.0832475132692129</v>
+        <v>0.08479740408105201</v>
       </c>
       <c r="O114" s="2" t="inlineStr">
         <is>
-          <t>market_above_ma60, avoid_chase, adx_trending</t>
+          <t>market_above_ma60, avoid_chase, kd_golden_cross</t>
         </is>
       </c>
     </row>
     <row r="115">
       <c r="A115" s="2" t="n">
-        <v>6890</v>
+        <v>6908</v>
       </c>
       <c r="B115" s="2" t="inlineStr">
         <is>
-          <t>來億-KY</t>
+          <t>宏碁遊戲-創</t>
         </is>
       </c>
       <c r="C115" s="2" t="n">
         <v/>
       </c>
       <c r="D115" s="2" t="n">
-        <v>179.9701783205616</v>
+        <v>183.0164824012788</v>
       </c>
       <c r="E115" s="2" t="n">
-        <v>168.5</v>
+        <v>32.8</v>
       </c>
       <c r="F115" s="2" t="inlineStr">
         <is>
@@ -6541,13 +6541,13 @@
         <v>0</v>
       </c>
       <c r="H115" s="2" t="n">
-        <v>41.287234344704</v>
+        <v>38.25126317374618</v>
       </c>
       <c r="I115" s="2" t="n">
-        <v>11.86301458870493</v>
+        <v>31.2457795599022</v>
       </c>
       <c r="J115" s="2" t="n">
-        <v>1.533637629554148</v>
+        <v>0.2051535797206257</v>
       </c>
       <c r="K115" s="2" t="n">
         <v>0</v>
@@ -6559,31 +6559,31 @@
         <v>-1</v>
       </c>
       <c r="N115" s="2" t="n">
-        <v>1.872216251345726</v>
+        <v>0.0832475132692129</v>
       </c>
       <c r="O115" s="2" t="inlineStr">
         <is>
-          <t>volume_break, market_above_ma60, avoid_chase</t>
+          <t>market_above_ma60, avoid_chase, adx_trending</t>
         </is>
       </c>
     </row>
     <row r="116">
       <c r="A116" s="2" t="n">
-        <v>6916</v>
+        <v>6890</v>
       </c>
       <c r="B116" s="2" t="inlineStr">
         <is>
-          <t>華凌</t>
+          <t>來億-KY</t>
         </is>
       </c>
       <c r="C116" s="2" t="n">
         <v/>
       </c>
       <c r="D116" s="2" t="n">
-        <v>167.6581768271423</v>
+        <v>179.9701783205616</v>
       </c>
       <c r="E116" s="2" t="n">
-        <v>18.6</v>
+        <v>168.5</v>
       </c>
       <c r="F116" s="2" t="inlineStr">
         <is>
@@ -6594,13 +6594,13 @@
         <v>0</v>
       </c>
       <c r="H116" s="2" t="n">
-        <v>46.72436108471069</v>
+        <v>41.287234344704</v>
       </c>
       <c r="I116" s="2" t="n">
-        <v>12.30942399130938</v>
+        <v>11.86301458870493</v>
       </c>
       <c r="J116" s="2" t="n">
-        <v>0.4866344054649537</v>
+        <v>1.533637629554148</v>
       </c>
       <c r="K116" s="2" t="n">
         <v>0</v>
@@ -6612,31 +6612,31 @@
         <v>-1</v>
       </c>
       <c r="N116" s="2" t="n">
-        <v>0.1003272439576099</v>
+        <v>1.872216251345726</v>
       </c>
       <c r="O116" s="2" t="inlineStr">
         <is>
-          <t>ema60_gt_ema120, market_above_ma60, avoid_chase</t>
+          <t>volume_break, market_above_ma60, avoid_chase</t>
         </is>
       </c>
     </row>
     <row r="117">
       <c r="A117" s="2" t="n">
-        <v>6947</v>
+        <v>6916</v>
       </c>
       <c r="B117" s="2" t="inlineStr">
         <is>
-          <t>台鎔科技</t>
+          <t>華凌</t>
         </is>
       </c>
       <c r="C117" s="2" t="n">
         <v/>
       </c>
       <c r="D117" s="2" t="n">
-        <v>163.3290837936911</v>
+        <v>167.6581768271423</v>
       </c>
       <c r="E117" s="2" t="n">
-        <v>72.3</v>
+        <v>18.6</v>
       </c>
       <c r="F117" s="2" t="inlineStr">
         <is>
@@ -6647,13 +6647,13 @@
         <v>0</v>
       </c>
       <c r="H117" s="2" t="n">
-        <v>38.84530136629972</v>
+        <v>46.72436108471069</v>
       </c>
       <c r="I117" s="2" t="n">
-        <v>16.22668937879958</v>
+        <v>12.30942399130938</v>
       </c>
       <c r="J117" s="2" t="n">
-        <v>0.4828318239338974</v>
+        <v>0.4866344054649537</v>
       </c>
       <c r="K117" s="2" t="n">
         <v>0</v>
@@ -6665,31 +6665,31 @@
         <v>-1</v>
       </c>
       <c r="N117" s="2" t="n">
-        <v>0.1838729249077837</v>
+        <v>0.1003272439576099</v>
       </c>
       <c r="O117" s="2" t="inlineStr">
         <is>
-          <t>market_above_ma60, avoid_chase, liquidity_ok</t>
+          <t>ema60_gt_ema120, market_above_ma60, avoid_chase</t>
         </is>
       </c>
     </row>
     <row r="118">
       <c r="A118" s="2" t="n">
-        <v>7753</v>
+        <v>6947</v>
       </c>
       <c r="B118" s="2" t="inlineStr">
         <is>
-          <t>星亞</t>
+          <t>台鎔科技</t>
         </is>
       </c>
       <c r="C118" s="2" t="n">
         <v/>
       </c>
       <c r="D118" s="2" t="n">
-        <v>146.8494454977195</v>
+        <v>163.3290837936911</v>
       </c>
       <c r="E118" s="2" t="n">
-        <v>37.5</v>
+        <v>72.3</v>
       </c>
       <c r="F118" s="2" t="inlineStr">
         <is>
@@ -6700,16 +6700,16 @@
         <v>0</v>
       </c>
       <c r="H118" s="2" t="n">
-        <v>40.28520062125639</v>
+        <v>38.84530136629972</v>
       </c>
       <c r="I118" s="2" t="n">
-        <v>10.56713667590755</v>
+        <v>16.22668937879958</v>
       </c>
       <c r="J118" s="2" t="n">
-        <v>0.9708165062904056</v>
+        <v>0.4828318239338974</v>
       </c>
       <c r="K118" s="2" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="L118" s="2" t="n">
         <v>0</v>
@@ -6718,31 +6718,31 @@
         <v>-1</v>
       </c>
       <c r="N118" s="2" t="n">
-        <v>0.0658653910454902</v>
+        <v>0.1838729249077837</v>
       </c>
       <c r="O118" s="2" t="inlineStr">
         <is>
-          <t>market_above_ma60, avoid_chase, kd_golden_cross</t>
+          <t>market_above_ma60, avoid_chase, liquidity_ok</t>
         </is>
       </c>
     </row>
     <row r="119">
       <c r="A119" s="2" t="n">
-        <v>7786</v>
+        <v>7753</v>
       </c>
       <c r="B119" s="2" t="inlineStr">
         <is>
-          <t>東方風能</t>
+          <t>星亞</t>
         </is>
       </c>
       <c r="C119" s="2" t="n">
         <v/>
       </c>
       <c r="D119" s="2" t="n">
-        <v>142.2424113012842</v>
+        <v>146.8494454977195</v>
       </c>
       <c r="E119" s="2" t="n">
-        <v>122.5</v>
+        <v>37.5</v>
       </c>
       <c r="F119" s="2" t="inlineStr">
         <is>
@@ -6753,16 +6753,16 @@
         <v>0</v>
       </c>
       <c r="H119" s="2" t="n">
-        <v>43.24719906643463</v>
+        <v>40.28520062125639</v>
       </c>
       <c r="I119" s="2" t="n">
-        <v>14.43973317235471</v>
+        <v>10.56713667590755</v>
       </c>
       <c r="J119" s="2" t="n">
-        <v>1.257092964439543</v>
+        <v>0.9708165062904056</v>
       </c>
       <c r="K119" s="2" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L119" s="2" t="n">
         <v>0</v>
@@ -6771,31 +6771,31 @@
         <v>-1</v>
       </c>
       <c r="N119" s="2" t="n">
-        <v>-0.08980499681302651</v>
+        <v>0.0658653910454902</v>
       </c>
       <c r="O119" s="2" t="inlineStr">
         <is>
-          <t>market_above_ma60, avoid_chase</t>
+          <t>market_above_ma60, avoid_chase, kd_golden_cross</t>
         </is>
       </c>
     </row>
     <row r="120">
       <c r="A120" s="2" t="n">
-        <v>7728</v>
+        <v>7786</v>
       </c>
       <c r="B120" s="2" t="inlineStr">
         <is>
-          <t>光焱科技</t>
+          <t>東方風能</t>
         </is>
       </c>
       <c r="C120" s="2" t="n">
         <v/>
       </c>
       <c r="D120" s="2" t="n">
-        <v>138.8525782114224</v>
+        <v>142.2424113012842</v>
       </c>
       <c r="E120" s="2" t="n">
-        <v>592</v>
+        <v>122.5</v>
       </c>
       <c r="F120" s="2" t="inlineStr">
         <is>
@@ -6806,13 +6806,13 @@
         <v>0</v>
       </c>
       <c r="H120" s="2" t="n">
-        <v>44.50836684562203</v>
+        <v>43.24719906643463</v>
       </c>
       <c r="I120" s="2" t="n">
-        <v>17.72213177716078</v>
+        <v>14.43973317235471</v>
       </c>
       <c r="J120" s="2" t="n">
-        <v>0.1827340653675267</v>
+        <v>1.257092964439543</v>
       </c>
       <c r="K120" s="2" t="n">
         <v>0</v>
@@ -6824,7 +6824,7 @@
         <v>-1</v>
       </c>
       <c r="N120" s="2" t="n">
-        <v>4.579428371383194</v>
+        <v>-0.08980499681302651</v>
       </c>
       <c r="O120" s="2" t="inlineStr">
         <is>
@@ -6834,21 +6834,21 @@
     </row>
     <row r="121">
       <c r="A121" s="2" t="n">
-        <v>6885</v>
+        <v>7728</v>
       </c>
       <c r="B121" s="2" t="inlineStr">
         <is>
-          <t>全福生技</t>
+          <t>光焱科技</t>
         </is>
       </c>
       <c r="C121" s="2" t="n">
         <v/>
       </c>
       <c r="D121" s="2" t="n">
-        <v>134.2626974369861</v>
+        <v>138.8525782114224</v>
       </c>
       <c r="E121" s="2" t="n">
-        <v>20.3</v>
+        <v>592</v>
       </c>
       <c r="F121" s="2" t="inlineStr">
         <is>
@@ -6859,13 +6859,13 @@
         <v>0</v>
       </c>
       <c r="H121" s="2" t="n">
-        <v>41.27900508691126</v>
+        <v>44.50836684562203</v>
       </c>
       <c r="I121" s="2" t="n">
-        <v>11.42680075144466</v>
+        <v>17.72213177716078</v>
       </c>
       <c r="J121" s="2" t="n">
-        <v>1.006218497096193</v>
+        <v>0.1827340653675267</v>
       </c>
       <c r="K121" s="2" t="n">
         <v>0</v>
@@ -6877,7 +6877,7 @@
         <v>-1</v>
       </c>
       <c r="N121" s="2" t="n">
-        <v>0.0157377152717733</v>
+        <v>4.579428371383194</v>
       </c>
       <c r="O121" s="2" t="inlineStr">
         <is>
@@ -6887,21 +6887,21 @@
     </row>
     <row r="122">
       <c r="A122" s="2" t="n">
-        <v>7740</v>
+        <v>6885</v>
       </c>
       <c r="B122" s="2" t="inlineStr">
         <is>
-          <t>熙特爾-創</t>
+          <t>全福生技</t>
         </is>
       </c>
       <c r="C122" s="2" t="n">
         <v/>
       </c>
       <c r="D122" s="2" t="n">
-        <v>124.7736182981662</v>
+        <v>134.2626974369861</v>
       </c>
       <c r="E122" s="2" t="n">
-        <v>141</v>
+        <v>20.3</v>
       </c>
       <c r="F122" s="2" t="inlineStr">
         <is>
@@ -6912,13 +6912,13 @@
         <v>0</v>
       </c>
       <c r="H122" s="2" t="n">
-        <v>42.90344778789896</v>
+        <v>41.27900508691126</v>
       </c>
       <c r="I122" s="2" t="n">
-        <v>17.20832335141327</v>
+        <v>11.42680075144466</v>
       </c>
       <c r="J122" s="2" t="n">
-        <v>0.6059034607016601</v>
+        <v>1.006218497096193</v>
       </c>
       <c r="K122" s="2" t="n">
         <v>0</v>
@@ -6930,7 +6930,7 @@
         <v>-1</v>
       </c>
       <c r="N122" s="2" t="n">
-        <v>-0.4099638962603154</v>
+        <v>0.0157377152717733</v>
       </c>
       <c r="O122" s="2" t="inlineStr">
         <is>
@@ -6940,21 +6940,21 @@
     </row>
     <row r="123">
       <c r="A123" s="2" t="n">
-        <v>6925</v>
+        <v>7740</v>
       </c>
       <c r="B123" s="2" t="inlineStr">
         <is>
-          <t>意藍</t>
+          <t>熙特爾-創</t>
         </is>
       </c>
       <c r="C123" s="2" t="n">
         <v/>
       </c>
       <c r="D123" s="2" t="n">
-        <v>123.4764912993379</v>
+        <v>124.7736182981662</v>
       </c>
       <c r="E123" s="2" t="n">
-        <v>52.5</v>
+        <v>141</v>
       </c>
       <c r="F123" s="2" t="inlineStr">
         <is>
@@ -6965,13 +6965,13 @@
         <v>0</v>
       </c>
       <c r="H123" s="2" t="n">
-        <v>40.5791876334731</v>
+        <v>42.90344778789896</v>
       </c>
       <c r="I123" s="2" t="n">
-        <v>13.79924073220903</v>
+        <v>17.20832335141327</v>
       </c>
       <c r="J123" s="2" t="n">
-        <v>0.966350199188354</v>
+        <v>0.6059034607016601</v>
       </c>
       <c r="K123" s="2" t="n">
         <v>0</v>
@@ -6983,7 +6983,7 @@
         <v>-1</v>
       </c>
       <c r="N123" s="2" t="n">
-        <v>0.4388814250122483</v>
+        <v>-0.4099638962603154</v>
       </c>
       <c r="O123" s="2" t="inlineStr">
         <is>
@@ -6993,21 +6993,21 @@
     </row>
     <row r="124">
       <c r="A124" s="2" t="n">
-        <v>7689</v>
+        <v>6925</v>
       </c>
       <c r="B124" s="2" t="inlineStr">
         <is>
-          <t>大鵬科CLMX</t>
+          <t>意藍</t>
         </is>
       </c>
       <c r="C124" s="2" t="n">
         <v/>
       </c>
       <c r="D124" s="2" t="n">
-        <v>121.8910333566369</v>
+        <v>123.4764912993379</v>
       </c>
       <c r="E124" s="2" t="n">
-        <v>173</v>
+        <v>52.5</v>
       </c>
       <c r="F124" s="2" t="inlineStr">
         <is>
@@ -7018,13 +7018,13 @@
         <v>0</v>
       </c>
       <c r="H124" s="2" t="n">
-        <v>30.55857914294411</v>
+        <v>40.5791876334731</v>
       </c>
       <c r="I124" s="2" t="n">
-        <v>31.37813133106843</v>
+        <v>13.79924073220903</v>
       </c>
       <c r="J124" s="2" t="n">
-        <v>0.4941161601743672</v>
+        <v>0.966350199188354</v>
       </c>
       <c r="K124" s="2" t="n">
         <v>0</v>
@@ -7036,31 +7036,31 @@
         <v>-1</v>
       </c>
       <c r="N124" s="2" t="n">
-        <v>1.799969222806659</v>
+        <v>0.4388814250122483</v>
       </c>
       <c r="O124" s="2" t="inlineStr">
         <is>
-          <t>market_above_ma60, adx_trending</t>
+          <t>market_above_ma60, avoid_chase</t>
         </is>
       </c>
     </row>
     <row r="125">
       <c r="A125" s="2" t="n">
-        <v>6923</v>
+        <v>7689</v>
       </c>
       <c r="B125" s="2" t="inlineStr">
         <is>
-          <t>中台</t>
+          <t>大鵬科CLMX</t>
         </is>
       </c>
       <c r="C125" s="2" t="n">
         <v/>
       </c>
       <c r="D125" s="2" t="n">
-        <v>107.2504571873362</v>
+        <v>121.8910333566369</v>
       </c>
       <c r="E125" s="2" t="n">
-        <v>76.09999999999999</v>
+        <v>173</v>
       </c>
       <c r="F125" s="2" t="inlineStr">
         <is>
@@ -7071,13 +7071,13 @@
         <v>0</v>
       </c>
       <c r="H125" s="2" t="n">
-        <v>48.91947851614185</v>
+        <v>30.55857914294411</v>
       </c>
       <c r="I125" s="2" t="n">
-        <v>9.141846616366037</v>
+        <v>31.37813133106843</v>
       </c>
       <c r="J125" s="2" t="n">
-        <v>0.5136415288972642</v>
+        <v>0.4941161601743672</v>
       </c>
       <c r="K125" s="2" t="n">
         <v>0</v>
@@ -7089,31 +7089,31 @@
         <v>-1</v>
       </c>
       <c r="N125" s="2" t="n">
-        <v>0.1198163255511222</v>
+        <v>1.799969222806659</v>
       </c>
       <c r="O125" s="2" t="inlineStr">
         <is>
-          <t>market_above_ma60, avoid_chase</t>
+          <t>market_above_ma60, adx_trending</t>
         </is>
       </c>
     </row>
     <row r="126">
       <c r="A126" s="2" t="n">
-        <v>6924</v>
+        <v>6923</v>
       </c>
       <c r="B126" s="2" t="inlineStr">
         <is>
-          <t>榮惠-KY創</t>
+          <t>中台</t>
         </is>
       </c>
       <c r="C126" s="2" t="n">
         <v/>
       </c>
       <c r="D126" s="2" t="n">
-        <v>92.08844267104328</v>
+        <v>107.2504571873362</v>
       </c>
       <c r="E126" s="2" t="n">
-        <v>115.5</v>
+        <v>76.09999999999999</v>
       </c>
       <c r="F126" s="2" t="inlineStr">
         <is>
@@ -7124,13 +7124,13 @@
         <v>0</v>
       </c>
       <c r="H126" s="2" t="n">
-        <v>52.96734899479101</v>
+        <v>48.91947851614185</v>
       </c>
       <c r="I126" s="2" t="n">
-        <v>16.7720153185608</v>
+        <v>9.141846616366037</v>
       </c>
       <c r="J126" s="2" t="n">
-        <v>0.2925884242877624</v>
+        <v>0.5136415288972642</v>
       </c>
       <c r="K126" s="2" t="n">
         <v>0</v>
@@ -7142,31 +7142,31 @@
         <v>-1</v>
       </c>
       <c r="N126" s="2" t="n">
-        <v>2.188413971435549</v>
+        <v>0.1198163255511222</v>
       </c>
       <c r="O126" s="2" t="inlineStr">
         <is>
-          <t>ema60_gt_ema120, market_above_ma60</t>
+          <t>market_above_ma60, avoid_chase</t>
         </is>
       </c>
     </row>
     <row r="127">
       <c r="A127" s="2" t="n">
-        <v>7760</v>
+        <v>6924</v>
       </c>
       <c r="B127" s="2" t="inlineStr">
         <is>
-          <t>享溫馨</t>
+          <t>榮惠-KY創</t>
         </is>
       </c>
       <c r="C127" s="2" t="n">
         <v/>
       </c>
       <c r="D127" s="2" t="n">
-        <v>91.4127226270659</v>
+        <v>92.08844267104328</v>
       </c>
       <c r="E127" s="2" t="n">
-        <v>33</v>
+        <v>115.5</v>
       </c>
       <c r="F127" s="2" t="inlineStr">
         <is>
@@ -7177,13 +7177,13 @@
         <v>0</v>
       </c>
       <c r="H127" s="2" t="n">
-        <v>42.80829996116454</v>
+        <v>52.96734899479101</v>
       </c>
       <c r="I127" s="2" t="n">
-        <v>12.30863597012752</v>
+        <v>16.7720153185608</v>
       </c>
       <c r="J127" s="2" t="n">
-        <v>0.8601537206972609</v>
+        <v>0.2925884242877624</v>
       </c>
       <c r="K127" s="2" t="n">
         <v>0</v>
@@ -7195,62 +7195,115 @@
         <v>-1</v>
       </c>
       <c r="N127" s="2" t="n">
-        <v>-0.1341137790138503</v>
+        <v>2.188413971435549</v>
       </c>
       <c r="O127" s="2" t="inlineStr">
         <is>
-          <t>market_above_ma60, avoid_chase</t>
+          <t>ema60_gt_ema120, market_above_ma60</t>
         </is>
       </c>
     </row>
     <row r="128">
       <c r="A128" s="2" t="n">
+        <v>7760</v>
+      </c>
+      <c r="B128" s="2" t="inlineStr">
+        <is>
+          <t>享溫馨</t>
+        </is>
+      </c>
+      <c r="C128" s="2" t="n">
+        <v/>
+      </c>
+      <c r="D128" s="2" t="n">
+        <v>91.4127226270659</v>
+      </c>
+      <c r="E128" s="2" t="n">
+        <v>33</v>
+      </c>
+      <c r="F128" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-14</t>
+        </is>
+      </c>
+      <c r="G128" s="2" t="b">
+        <v>0</v>
+      </c>
+      <c r="H128" s="2" t="n">
+        <v>42.80829996116454</v>
+      </c>
+      <c r="I128" s="2" t="n">
+        <v>12.30863597012752</v>
+      </c>
+      <c r="J128" s="2" t="n">
+        <v>0.8601537206972609</v>
+      </c>
+      <c r="K128" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="L128" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="M128" s="2" t="n">
+        <v>-1</v>
+      </c>
+      <c r="N128" s="2" t="n">
+        <v>-0.1341137790138503</v>
+      </c>
+      <c r="O128" s="2" t="inlineStr">
+        <is>
+          <t>market_above_ma60, avoid_chase</t>
+        </is>
+      </c>
+    </row>
+    <row r="129">
+      <c r="A129" s="2" t="n">
         <v>6934</v>
       </c>
-      <c r="B128" s="2" t="inlineStr">
+      <c r="B129" s="2" t="inlineStr">
         <is>
           <t>心誠鎂</t>
         </is>
       </c>
-      <c r="C128" s="2" t="n">
-        <v/>
-      </c>
-      <c r="D128" s="2" t="n">
+      <c r="C129" s="2" t="n">
+        <v/>
+      </c>
+      <c r="D129" s="2" t="n">
         <v>90.54901949610382</v>
       </c>
-      <c r="E128" s="2" t="n">
+      <c r="E129" s="2" t="n">
         <v>72.3</v>
       </c>
-      <c r="F128" s="2" t="inlineStr">
-        <is>
-          <t>2026-08-14</t>
-        </is>
-      </c>
-      <c r="G128" s="2" t="b">
-        <v>0</v>
-      </c>
-      <c r="H128" s="2" t="n">
+      <c r="F129" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-14</t>
+        </is>
+      </c>
+      <c r="G129" s="2" t="b">
+        <v>0</v>
+      </c>
+      <c r="H129" s="2" t="n">
         <v>44.30663008198438</v>
       </c>
-      <c r="I128" s="2" t="n">
+      <c r="I129" s="2" t="n">
         <v>17.93612213130106</v>
       </c>
-      <c r="J128" s="2" t="n">
+      <c r="J129" s="2" t="n">
         <v>1.155005587336816</v>
       </c>
-      <c r="K128" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="L128" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="M128" s="2" t="n">
-        <v>-1</v>
-      </c>
-      <c r="N128" s="2" t="n">
+      <c r="K129" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="L129" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="M129" s="2" t="n">
+        <v>-1</v>
+      </c>
+      <c r="N129" s="2" t="n">
         <v>-0.5582836820414379</v>
       </c>
-      <c r="O128" s="2" t="inlineStr">
+      <c r="O129" s="2" t="inlineStr">
         <is>
           <t>market_above_ma60, avoid_chase</t>
         </is>

</xml_diff>